<commit_message>
Fix dependency cleanup and tighten dashboard query consistency
</commit_message>
<xml_diff>
--- a/docs/跑批监控接口出入参文档.xlsx
+++ b/docs/跑批监控接口出入参文档.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="15660"/>
+    <workbookView windowHeight="15660" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="接口清单" sheetId="1" r:id="rId1"/>
@@ -2624,8 +2624,8 @@
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="36.8653846153846" customWidth="1"/>
+    <col min="1" max="1" width="43.2692307692308" customWidth="1"/>
+    <col min="2" max="2" width="71.4711538461538" customWidth="1"/>
     <col min="3" max="3" width="24" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>